<commit_message>
full first draft of accessibility audits
</commit_message>
<xml_diff>
--- a/input_info/harvest/Cryosat Accessions.xlsx
+++ b/input_info/harvest/Cryosat Accessions.xlsx
@@ -622,6 +622,10 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="4" max="4" width="33.13"/>
+    <col customWidth="1" min="5" max="5" width="26.0"/>
+    <col customWidth="1" min="6" max="6" width="17.0"/>
+    <col customWidth="1" min="7" max="7" width="46.0"/>
+    <col customWidth="1" min="8" max="8" width="64.0"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -651,6 +655,26 @@
       <c r="D3" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SAC IDs (JASADCP)</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JASADCP accession</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NCEI link</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archive status (resolved Sept 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
@@ -659,11 +683,33 @@
       <c r="B4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>7</v>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0309821</t>
+        </is>
       </c>
       <c r="D4" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02499</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0309821</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived twice: direct submission 0309821 and JASADCP batch 0223175</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -673,11 +719,23 @@
       <c r="B5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>10</v>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0309822</t>
+        </is>
       </c>
       <c r="D5" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0309822</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -687,11 +745,23 @@
       <c r="B6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>12</v>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0309820</t>
+        </is>
       </c>
       <c r="D6" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0309820</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -701,11 +771,23 @@
       <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>14</v>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0308264</t>
+        </is>
       </c>
       <c r="D7" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0308264</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -715,11 +797,23 @@
       <c r="B8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>16</v>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0308398</t>
+        </is>
       </c>
       <c r="D8" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0308398</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -729,11 +823,23 @@
       <c r="B9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>18</v>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0308524</t>
+        </is>
       </c>
       <c r="D9" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0308524</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -743,11 +849,23 @@
       <c r="B10" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>20</v>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0308564</t>
+        </is>
       </c>
       <c r="D10" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0308564</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -757,11 +875,33 @@
       <c r="B11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>23</v>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0313189</t>
+        </is>
       </c>
       <c r="D11" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02506 02507 02508</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0313189</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived twice: direct submission 0313189 and JASADCP batch 0223175</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -771,11 +911,33 @@
       <c r="B12" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="10" t="s">
-        <v>25</v>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0313191</t>
+        </is>
       </c>
       <c r="D12" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02509 02510 02511</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0313191</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived twice: direct submission 0313191 and JASADCP batch 0223175</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -785,11 +947,33 @@
       <c r="B13" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="10" t="s">
-        <v>27</v>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0313190</t>
+        </is>
       </c>
       <c r="D13" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02512 02513 02514</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0313190</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived twice: direct submission 0313190 and JASADCP batch 0223175</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -799,8 +983,36 @@
       <c r="B14" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Published</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02515 02516 02517</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0223175</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived in JASADCP batch 0223175 - found Sept 2026, not previously recorded</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="s">
@@ -809,11 +1021,23 @@
       <c r="B15" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="4">
-        <v>314052.0</v>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0314052</t>
+        </is>
       </c>
       <c r="D15" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0314052</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -823,11 +1047,23 @@
       <c r="B16" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="4">
-        <v>314053.0</v>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0314053</t>
+        </is>
       </c>
       <c r="D16" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0314053</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -837,8 +1073,36 @@
       <c r="B17" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Published</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02519 02520</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0223175</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived in JASADCP batch 0223175 - found Sept 2026, not previously recorded</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="s">
@@ -847,11 +1111,33 @@
       <c r="B18" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="4">
-        <v>314506.0</v>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0314506</t>
+        </is>
       </c>
       <c r="D18" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02521 02522</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0314506</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived twice: direct submission 0314506 and JASADCP batch 0223175</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -863,6 +1149,11 @@
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="s">
@@ -871,8 +1162,36 @@
       <c r="B20" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Published</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02534 02535</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0223175</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived in JASADCP batch 0223175 - found Sept 2026, not previously recorded</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="s">
@@ -881,8 +1200,36 @@
       <c r="B21" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Published</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02523 02524 02525</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0223175</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived in JASADCP batch 0223175 - found Sept 2026, not previously recorded</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="s">
@@ -891,8 +1238,36 @@
       <c r="B22" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Published</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02526 02527 02528</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0223175</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived in JASADCP batch 0223175 - found Sept 2026, not previously recorded</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="s">
@@ -901,8 +1276,36 @@
       <c r="B23" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Published</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02540 02541</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0223175</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived in JASADCP batch 0223175 - found Sept 2026, not previously recorded</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="s">
@@ -911,8 +1314,36 @@
       <c r="B24" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Published</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02542 02543</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0223175</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived in JASADCP batch 0223175 - found Sept 2026, not previously recorded</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="s">
@@ -921,8 +1352,36 @@
       <c r="B25" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Published</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02536 02537</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0223175</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived in JASADCP batch 0223175 - found Sept 2026, not previously recorded</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="s">
@@ -931,8 +1390,36 @@
       <c r="B26" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Published</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02538 02539</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0223175</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived in JASADCP batch 0223175 - found Sept 2026, not previously recorded</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="s">
@@ -941,8 +1428,36 @@
       <c r="B27" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Published</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02546 02547 02548</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0223175</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived in JASADCP batch 0223175 - found Sept 2026, not previously recorded</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="s">
@@ -953,6 +1468,11 @@
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="s">
@@ -961,8 +1481,36 @@
       <c r="B29" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Published</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02551 02552</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0223175</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived in JASADCP batch 0223175 - found Sept 2026, not previously recorded</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="s">
@@ -971,8 +1519,36 @@
       <c r="B30" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Published</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02553 02554</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0223175</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived in JASADCP batch 0223175 - found Sept 2026, not previously recorded</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="s">
@@ -981,8 +1557,36 @@
       <c r="B31" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Published</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02555 02556</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0223175</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived in JASADCP batch 0223175 - found Sept 2026, not previously recorded</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="s">
@@ -993,6 +1597,11 @@
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="s">
@@ -1003,6 +1612,11 @@
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="s">
@@ -1011,8 +1625,36 @@
       <c r="B34" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Published</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02557 02558</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0223175</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived in JASADCP batch 0223175 - found Sept 2026, not previously recorded</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="s">
@@ -1021,8 +1663,36 @@
       <c r="B35" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Published</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">02559 02560</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0223175</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0223175</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archived in JASADCP batch 0223175 - found Sept 2026, not previously recorded</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="s">
@@ -1031,11 +1701,23 @@
       <c r="B36" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C36" s="7" t="s">
-        <v>60</v>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0306284</t>
+        </is>
       </c>
       <c r="D36" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0306284</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -1045,11 +1727,23 @@
       <c r="B37" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C37" s="7" t="s">
-        <v>62</v>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0306335</t>
+        </is>
       </c>
       <c r="D37" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0306335</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1059,11 +1753,23 @@
       <c r="B38" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C38" s="7" t="s">
-        <v>64</v>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0307837</t>
+        </is>
       </c>
       <c r="D38" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0307837</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -1073,11 +1779,23 @@
       <c r="B39" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="C39" s="7" t="s">
-        <v>67</v>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0314508</t>
+        </is>
       </c>
       <c r="D39" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0314508</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -1087,11 +1805,23 @@
       <c r="B40" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="C40" s="7" t="s">
-        <v>69</v>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0316807</t>
+        </is>
       </c>
       <c r="D40" s="4" t="s">
         <v>70</v>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0316807</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -1103,6 +1833,11 @@
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="s">
@@ -1111,11 +1846,23 @@
       <c r="B42" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C42" s="4">
-        <v>314048.0</v>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0314048</t>
+        </is>
       </c>
       <c r="D42" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0314048</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -1125,11 +1872,23 @@
       <c r="B43" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="C43" s="4">
-        <v>314054.0</v>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0314054</t>
+        </is>
       </c>
       <c r="D43" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0314054</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -1139,11 +1898,23 @@
       <c r="B44" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C44" s="4">
-        <v>314049.0</v>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0314049</t>
+        </is>
       </c>
       <c r="D44" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.ncei.noaa.gov/archive/accession/0314049</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct submission to NCEI</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -1155,6 +1926,11 @@
       </c>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="s">
@@ -1165,6 +1941,11 @@
       </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="s">
@@ -1175,6 +1956,11 @@
       </c>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="s">
@@ -1185,6 +1971,11 @@
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="s">
@@ -1195,6 +1986,11 @@
       </c>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="s">
@@ -1205,6 +2001,11 @@
       </c>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="s">
@@ -1215,6 +2016,11 @@
       </c>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="s">
@@ -1225,6 +2031,11 @@
       </c>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="s">
@@ -1235,6 +2046,11 @@
       </c>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="s">
@@ -1245,6 +2061,11 @@
       </c>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="s">
@@ -1255,6 +2076,11 @@
       </c>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="s">
@@ -1265,6 +2091,11 @@
       </c>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="s">
@@ -1275,6 +2106,11 @@
       </c>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="s">
@@ -1285,6 +2121,11 @@
       </c>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="s">
@@ -1295,6 +2136,11 @@
       </c>
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="s">
@@ -1305,6 +2151,11 @@
       </c>
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="9" t="s">
@@ -1315,6 +2166,11 @@
       </c>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not archived: absent from the JASADCP inventory and from NCEI</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2"/>
@@ -7002,6 +7858,42 @@
     <hyperlink r:id="rId19" ref="B42"/>
     <hyperlink r:id="rId20" ref="B43"/>
     <hyperlink r:id="rId21" ref="B44"/>
+    <hyperlink r:id="rId23" ref="G4"/>
+    <hyperlink r:id="rId24" ref="G5"/>
+    <hyperlink r:id="rId25" ref="G6"/>
+    <hyperlink r:id="rId26" ref="G7"/>
+    <hyperlink r:id="rId27" ref="G8"/>
+    <hyperlink r:id="rId28" ref="G9"/>
+    <hyperlink r:id="rId29" ref="G10"/>
+    <hyperlink r:id="rId30" ref="G11"/>
+    <hyperlink r:id="rId31" ref="G12"/>
+    <hyperlink r:id="rId32" ref="G13"/>
+    <hyperlink r:id="rId33" ref="G14"/>
+    <hyperlink r:id="rId34" ref="G15"/>
+    <hyperlink r:id="rId35" ref="G16"/>
+    <hyperlink r:id="rId36" ref="G17"/>
+    <hyperlink r:id="rId37" ref="G18"/>
+    <hyperlink r:id="rId38" ref="G20"/>
+    <hyperlink r:id="rId39" ref="G21"/>
+    <hyperlink r:id="rId40" ref="G22"/>
+    <hyperlink r:id="rId41" ref="G23"/>
+    <hyperlink r:id="rId42" ref="G24"/>
+    <hyperlink r:id="rId43" ref="G25"/>
+    <hyperlink r:id="rId44" ref="G26"/>
+    <hyperlink r:id="rId45" ref="G27"/>
+    <hyperlink r:id="rId46" ref="G29"/>
+    <hyperlink r:id="rId47" ref="G30"/>
+    <hyperlink r:id="rId48" ref="G31"/>
+    <hyperlink r:id="rId49" ref="G34"/>
+    <hyperlink r:id="rId50" ref="G35"/>
+    <hyperlink r:id="rId51" ref="G36"/>
+    <hyperlink r:id="rId52" ref="G37"/>
+    <hyperlink r:id="rId53" ref="G38"/>
+    <hyperlink r:id="rId54" ref="G39"/>
+    <hyperlink r:id="rId55" ref="G40"/>
+    <hyperlink r:id="rId56" ref="G42"/>
+    <hyperlink r:id="rId57" ref="G43"/>
+    <hyperlink r:id="rId58" ref="G44"/>
   </hyperlinks>
   <drawing r:id="rId22"/>
 </worksheet>

</xml_diff>